<commit_message>
fix: O Bot agora executa pelo comando de 'python bot.py'
</commit_message>
<xml_diff>
--- a/data/samples/inspecao_lotes_dia_teste.xlsx
+++ b/data/samples/inspecao_lotes_dia_teste.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="111">
   <si>
     <t xml:space="preserve">PLANILHA DE INSPEÇÃO DE LOTES  ·  REFERÊNCIA: 14/06/2026  ·  LG Electronics — Qualidade</t>
   </si>
@@ -166,9 +166,6 @@
   </si>
   <si>
     <t xml:space="preserve">MON32-4K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Falha no painel de controle</t>
   </si>
   <si>
     <t xml:space="preserve">LG-2026-00110</t>
@@ -1309,17 +1306,17 @@
       <c r="E12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="10"/>
+      <c r="F12" s="10" t="s">
+        <v>21</v>
+      </c>
       <c r="G12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>48</v>
-      </c>
+      <c r="H12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>11</v>
@@ -1343,10 +1340,10 @@
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>19</v>
@@ -1367,7 +1364,7 @@
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>37</v>
@@ -1379,7 +1376,7 @@
         <v>13</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>35</v>
@@ -1391,7 +1388,7 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>18</v>
@@ -1415,7 +1412,7 @@
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>27</v>
@@ -1436,12 +1433,12 @@
         <v>16</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>23</v>
@@ -1459,13 +1456,13 @@
         <v>21</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>45</v>
@@ -1486,12 +1483,12 @@
         <v>16</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>33</v>
@@ -1515,7 +1512,7 @@
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>37</v>
@@ -1527,7 +1524,7 @@
         <v>20</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>35</v>
@@ -1536,12 +1533,12 @@
         <v>16</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>42</v>
@@ -1565,7 +1562,7 @@
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>11</v>
@@ -1589,7 +1586,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>47</v>
@@ -1613,7 +1610,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>27</v>
@@ -1637,10 +1634,10 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>19</v>
@@ -1660,7 +1657,9 @@
       <c r="H26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10"/>
+      <c r="A27" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="B27" s="7" t="s">
         <v>45</v>
       </c>
@@ -1683,7 +1682,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>18</v>
@@ -1704,18 +1703,18 @@
         <v>16</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
       <c r="E29" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
@@ -1723,7 +1722,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
@@ -1735,11 +1734,11 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D32" s="15"/>
       <c r="E32" s="15"/>
@@ -1749,11 +1748,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D33" s="15"/>
       <c r="E33" s="15"/>
@@ -1763,11 +1762,11 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B34" s="17"/>
       <c r="C34" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D34" s="15"/>
       <c r="E34" s="15"/>
@@ -1777,11 +1776,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B35" s="18"/>
       <c r="C35" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="15"/>
@@ -1831,7 +1830,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1842,13 +1841,13 @@
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1859,10 +1858,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1873,10 +1872,10 @@
         <v>18</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1887,10 +1886,10 @@
         <v>27</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1901,10 +1900,10 @@
         <v>33</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1915,10 +1914,10 @@
         <v>37</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1929,10 +1928,10 @@
         <v>42</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1943,10 +1942,10 @@
         <v>45</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1957,225 +1956,225 @@
         <v>47</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>51</v>
-      </c>
       <c r="C12" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="20" t="s">
         <v>37</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" s="22" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="20" t="s">
         <v>27</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" s="20" t="s">
         <v>45</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="22" t="s">
         <v>33</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="20" t="s">
         <v>37</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" s="22" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="20" t="s">
         <v>11</v>
       </c>
       <c r="C21" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="22" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>27</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B27" s="24"/>
       <c r="C27" s="24"/>
@@ -2214,7 +2213,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -2224,7 +2223,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -2234,22 +2233,22 @@
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2504,7 +2503,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B30" s="13"/>
       <c r="C30" s="30"/>
@@ -2514,7 +2513,7 @@
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B31" s="31"/>
       <c r="C31" s="31"/>
@@ -2524,7 +2523,7 @@
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B32" s="31"/>
       <c r="C32" s="31"/>
@@ -2534,7 +2533,7 @@
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B33" s="31"/>
       <c r="C33" s="31"/>
@@ -2544,7 +2543,7 @@
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="31" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
@@ -2554,7 +2553,7 @@
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B35" s="31"/>
       <c r="C35" s="31"/>
@@ -2564,7 +2563,7 @@
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B36" s="31"/>
       <c r="C36" s="31"/>
@@ -2574,7 +2573,7 @@
     </row>
     <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="31" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B37" s="31"/>
       <c r="C37" s="31"/>
@@ -2584,7 +2583,7 @@
     </row>
     <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>

</xml_diff>